<commit_message>
ATUALIZAÇÃO DO CONCEITUAL CRIAÇAÕ TESTE SCRIPT E O DICIONARIO
</commit_message>
<xml_diff>
--- a/docs/modelo_dicionario_de_dados.xlsx
+++ b/docs/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="123">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Chave prmaria de identificação do funcionario</t>
   </si>
   <si>
-    <t xml:space="preserve">nome </t>
+    <t xml:space="preserve">nome_funcionario</t>
   </si>
   <si>
     <t xml:space="preserve">TEXT</t>
@@ -111,28 +111,88 @@
     <t xml:space="preserve">DATE</t>
   </si>
   <si>
-    <t xml:space="preserve">id_status</t>
+    <t xml:space="preserve">status</t>
   </si>
   <si>
     <t xml:space="preserve">Id-cargo</t>
   </si>
   <si>
+    <t xml:space="preserve">cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_cargo</t>
+  </si>
+  <si>
     <t xml:space="preserve">cliente</t>
   </si>
   <si>
     <t xml:space="preserve">Chave prmaria de identificação do cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">nome_cliente</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo nome do cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">criação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">telefone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_cargo</t>
+  </si>
+  <si>
     <t xml:space="preserve">equipamento</t>
   </si>
   <si>
     <t xml:space="preserve">Chave prmaria de identificação do equipamento</t>
   </si>
   <si>
+    <t xml:space="preserve">id_modelo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Campo nome do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">imei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modelo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_tipo</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -484,13 +544,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -543,6 +607,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -809,12 +877,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26"/>
@@ -823,173 +891,161 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="10" t="s">
+      <c r="H10" s="8"/>
+      <c r="I10" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13" t="s">
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="12"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="14" t="s">
+      <c r="G11" s="13"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="0"/>
-      <c r="E12" s="0"/>
-      <c r="F12" s="0"/>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="0"/>
-      <c r="E14" s="0"/>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
+      <c r="A15" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>19</v>
+      </c>
       <c r="D15" s="0"/>
       <c r="E15" s="0"/>
       <c r="F15" s="0"/>
@@ -998,548 +1054,718 @@
       <c r="I15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="10"/>
+      <c r="A16" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="14"/>
+      <c r="A17" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="0"/>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="10"/>
+      <c r="A18" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9" t="s">
+      <c r="D19" s="10"/>
+      <c r="E19" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="10" t="s">
-        <v>32</v>
+      <c r="H19" s="8"/>
+      <c r="I19" s="11" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="12" t="s">
+      <c r="A20" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13" t="s">
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G20" s="12"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="14" t="s">
+      <c r="G20" s="13"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="15"/>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="0"/>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0"/>
+      <c r="G23" s="0"/>
+      <c r="H23" s="0"/>
+      <c r="I23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="0"/>
+      <c r="E24" s="0"/>
+      <c r="F24" s="0"/>
+      <c r="G24" s="0"/>
+      <c r="H24" s="0"/>
+      <c r="I24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="0"/>
+      <c r="E25" s="0"/>
+      <c r="F25" s="0"/>
+      <c r="G25" s="0"/>
+      <c r="H25" s="0"/>
+      <c r="I25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="0"/>
+      <c r="E26" s="0"/>
+      <c r="F26" s="0"/>
+      <c r="G26" s="0"/>
+      <c r="H26" s="0"/>
+      <c r="I26" s="0"/>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="0"/>
+      <c r="E27" s="0"/>
+      <c r="F27" s="0"/>
+      <c r="G27" s="0"/>
+      <c r="H27" s="0"/>
+      <c r="I27" s="0"/>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C28" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9" t="s">
+      <c r="D28" s="10"/>
+      <c r="E28" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F28" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G28" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13" t="s">
+      <c r="H28" s="8"/>
+      <c r="I28" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G22" s="12"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="14"/>
-    </row>
-    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="14"/>
-    </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="10"/>
-    </row>
-    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="14"/>
-    </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="10"/>
-    </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="14"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="15" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="10"/>
+      <c r="A30" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="14"/>
+      <c r="A31" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="10"/>
+      <c r="A32" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="0"/>
+      <c r="E32" s="0"/>
+      <c r="F32" s="0"/>
+      <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
+      <c r="I32" s="0"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="14"/>
+      <c r="A33" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="0"/>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="10"/>
+      <c r="A34" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="14"/>
+      <c r="A35" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="10"/>
+      <c r="A36" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" s="9"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="14"/>
+      <c r="A37" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="16"/>
+      <c r="D37" s="0"/>
+      <c r="E37" s="0"/>
+      <c r="F37" s="0"/>
+      <c r="G37" s="0"/>
+      <c r="H37" s="0"/>
+      <c r="I37" s="0"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="10"/>
+      <c r="A38" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="16"/>
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
+      <c r="F38" s="0"/>
+      <c r="G38" s="0"/>
+      <c r="H38" s="0"/>
+      <c r="I38" s="0"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="14"/>
+      <c r="A39" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C39" s="16"/>
+      <c r="D39" s="0"/>
+      <c r="E39" s="0"/>
+      <c r="F39" s="0"/>
+      <c r="G39" s="0"/>
+      <c r="H39" s="0"/>
+      <c r="I39" s="0"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="10"/>
+      <c r="A40" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="16"/>
+      <c r="D40" s="0"/>
+      <c r="E40" s="0"/>
+      <c r="F40" s="0"/>
+      <c r="G40" s="0"/>
+      <c r="H40" s="0"/>
+      <c r="I40" s="0"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="14"/>
+      <c r="A41" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C41" s="16"/>
+      <c r="D41" s="0"/>
+      <c r="E41" s="0"/>
+      <c r="F41" s="0"/>
+      <c r="G41" s="0"/>
+      <c r="H41" s="0"/>
+      <c r="I41" s="0"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="7"/>
-      <c r="I42" s="10"/>
+      <c r="A42" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C42" s="16"/>
+      <c r="D42" s="0"/>
+      <c r="E42" s="0"/>
+      <c r="F42" s="0"/>
+      <c r="G42" s="0"/>
+      <c r="H42" s="0"/>
+      <c r="I42" s="0"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="14"/>
+      <c r="A43" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="0"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="0"/>
+      <c r="E43" s="0"/>
+      <c r="F43" s="0"/>
+      <c r="G43" s="0"/>
+      <c r="H43" s="0"/>
+      <c r="I43" s="0"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="7"/>
-      <c r="I44" s="10"/>
+      <c r="A44" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="0"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="0"/>
+      <c r="E44" s="0"/>
+      <c r="F44" s="0"/>
+      <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="14"/>
+      <c r="A45" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="16"/>
+      <c r="D45" s="0"/>
+      <c r="E45" s="0"/>
+      <c r="F45" s="0"/>
+      <c r="G45" s="0"/>
+      <c r="H45" s="0"/>
+      <c r="I45" s="0"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="10"/>
+      <c r="A46" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="9"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="14"/>
+      <c r="A47" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47" s="13"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="15"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7"/>
-      <c r="B48" s="7"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="7"/>
-      <c r="I48" s="10"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="12"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="14"/>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="10"/>
+      <c r="A50" s="8"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="11"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="12"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="14"/>
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="15"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="10"/>
+      <c r="A52" s="8"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="14"/>
+      <c r="A53" s="12"/>
+      <c r="B53" s="12"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="7"/>
-      <c r="I54" s="10"/>
+      <c r="A54" s="8"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="11"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="14"/>
+      <c r="A55" s="12"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="12"/>
+      <c r="I55" s="15"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="7"/>
-      <c r="I56" s="10"/>
+      <c r="A56" s="8"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="11"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="14"/>
+      <c r="A57" s="12"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="13"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="14"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="15"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7"/>
-      <c r="B58" s="7"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="7"/>
-      <c r="I58" s="10"/>
+      <c r="A58" s="8"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="8"/>
+      <c r="I58" s="11"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="11"/>
-      <c r="I59" s="14"/>
+      <c r="A59" s="12"/>
+      <c r="B59" s="12"/>
+      <c r="C59" s="13"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="14"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="15"/>
+    </row>
+    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="8"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="11"/>
+    </row>
+    <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12"/>
+      <c r="B61" s="12"/>
+      <c r="C61" s="13"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="14"/>
+      <c r="G61" s="13"/>
+      <c r="H61" s="12"/>
+      <c r="I61" s="15"/>
+    </row>
+    <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="8"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="10"/>
+      <c r="E62" s="10"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="9"/>
+      <c r="H62" s="8"/>
+      <c r="I62" s="11"/>
+    </row>
+    <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="12"/>
+      <c r="B63" s="12"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14"/>
+      <c r="G63" s="13"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="15"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C16:C59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C19:C22 C28:C31 C34:C36 C46:C63" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E16:E59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E19:E22 E28:E31 E34:E36 E46:E63" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F11 F16:F59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F11 F19:F22 F28:F31 F34:F36 F46:F63" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1573,362 +1799,362 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>37</v>
+      <c r="A1" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>38</v>
+      <c r="A2" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>40</v>
+      <c r="A4" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>42</v>
+      <c r="A5" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>44</v>
+      <c r="A6" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>46</v>
+      <c r="A7" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>48</v>
+      <c r="A8" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>50</v>
+      <c r="A9" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>52</v>
+      <c r="A10" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>54</v>
+      <c r="A11" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>56</v>
+      <c r="A12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>57</v>
+      <c r="A14" s="19" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="B16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I16" s="6" t="s">
+      <c r="G16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="A17" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="13" t="s">
+      <c r="D17" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>67</v>
+      <c r="F17" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>72</v>
+      <c r="A18" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>74</v>
+      <c r="A19" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="8" t="s">
+      <c r="A20" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>76</v>
+      <c r="D20" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>80</v>
+      <c r="A21" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="B22" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H22" s="7" t="s">
+      <c r="D22" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="E22" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="10" t="s">
         <v>84</v>
       </c>
+      <c r="G22" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G23" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="H23" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="H23" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E25" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>93</v>
+      <c r="F25" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1958,39 +2184,39 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2000,7 +2226,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,17 +2236,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cRIAÇÃO DE TABELAS ORDEM DE SERVICOS
</commit_message>
<xml_diff>
--- a/docs/modelo_dicionario_de_dados.xlsx
+++ b/docs/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="277">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -334,6 +334,333 @@
   </si>
   <si>
     <t xml:space="preserve">Cargo do funcionário que cadastrou o tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da categoria de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome da categoria de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data de cadastro da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status da categoria (1=Ativo, 0=Inativo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcionário que cadastrou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do funcionário no cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome ou descrição do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço padrão do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tempo_trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tempo estimado de trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data de cadastro do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status do serviço (1=Ativo, 0=Inativo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da ordem de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliente da ordem de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipamento (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipamento em manutenção</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora de abertura da OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_fechamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora de fechamento da OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_situacao_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status/Situação atual da OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">descricao_problema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrição do problema relatado pelo cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">defeito_constatado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defeito real constatado pelo técnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor total da ordem de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forma_pagamento (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forma de pagamento utilizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico responsável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do técnico responsável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_servicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária do serviço na OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_ordem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem de serviço associada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servico (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serviço realizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_cobrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor cobrado pelo serviço nesta OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico que executou o serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do técnico que executou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_adicao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data de adição do serviço na OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome da situação (ex: Aberta, Em Andamento, Concluída)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status ativo (1) ou inativo (0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária do histórico de situação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem de serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Situação registrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_atualizacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data da alteração do status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcionário que alterou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do funcionário no momento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da forma de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrição (ex: Dinheiro, Cartão, PIX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da categoria da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome da categoria (ex: Telas, Baterias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data de cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pecas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_categoria_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria_peca (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria pertencente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrição/Nome da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_venda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço de venda da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">estoque_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade em estoque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_pecas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da peça na OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pecas (id)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peça utilizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade de peças utilizadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_unitario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor cobrado pela peça nesta OS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico que aplicou a peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do técnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data de adição da peça na OS</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -1012,7 +1339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I137"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -1022,7 +1349,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="49.05"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1325,15 +1652,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0"/>
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
+      <c r="C18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -1539,15 +1858,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0"/>
-      <c r="B26" s="0"/>
-      <c r="C26" s="0"/>
-      <c r="D26" s="0"/>
-      <c r="E26" s="0"/>
-      <c r="F26" s="0"/>
-      <c r="G26" s="0"/>
-      <c r="H26" s="0"/>
-      <c r="I26" s="0"/>
+      <c r="C26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
@@ -1869,61 +2180,35 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>81</v>
-      </c>
+      <c r="C38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>22</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>20</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1931,7 +2216,7 @@
         <v>80</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>26</v>
@@ -1946,13 +2231,13 @@
         <v>22</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>20</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1960,10 +2245,10 @@
         <v>80</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>20</v>
@@ -1974,14 +2259,14 @@
       <c r="F41" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G41" s="1" t="n">
-        <v>1</v>
+      <c r="G41" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>20</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1989,7 +2274,7 @@
         <v>80</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>19</v>
@@ -1998,19 +2283,19 @@
         <v>20</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>20</v>
+      <c r="G42" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2018,7 +2303,7 @@
         <v>80</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>19</v>
@@ -2036,18 +2321,18 @@
         <v>20</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="C44" s="16" t="s">
         <v>19</v>
@@ -2056,77 +2341,51 @@
         <v>20</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>22</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="C45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I46" s="11" t="s">
-        <v>92</v>
+        <v>18</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2134,94 +2393,94 @@
         <v>88</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I48" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C47" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G47" s="13" t="n">
+      <c r="C49" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G49" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H47" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I47" s="15" t="s">
+      <c r="H49" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I49" s="15" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F48" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="I48" s="11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="F49" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G49" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H49" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="I49" s="15" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>19</v>
@@ -2230,198 +2489,234 @@
         <v>20</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="F50" s="10" t="s">
         <v>22</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="I51" s="15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="15"/>
+    </row>
+    <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B53" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H53" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="C54" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D51" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G51" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I51" s="15" t="s">
+      <c r="D54" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G54" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I54" s="15" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="8" t="s">
+    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="B55" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C55" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G52" s="9" t="s">
+      <c r="D55" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G55" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="H52" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I52" s="11" t="s">
+      <c r="H55" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I55" s="11" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12" t="s">
+    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B56" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C53" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D53" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F53" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G53" s="13" t="n">
+      <c r="C56" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G56" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I53" s="15" t="s">
+      <c r="H56" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" s="15" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8" t="s">
+    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B57" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C54" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E54" s="10" t="s">
+      <c r="C57" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E57" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F54" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="H54" s="8" t="s">
+      <c r="F57" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H57" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="I54" s="11" t="s">
+      <c r="I57" s="11" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="s">
+    <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B55" s="12" t="s">
+      <c r="B58" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="C55" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D55" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E55" s="14" t="s">
+      <c r="C58" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E58" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F55" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G55" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H55" s="12" t="s">
+      <c r="F58" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G58" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H58" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="I55" s="15" t="s">
+      <c r="I58" s="15" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="8"/>
-      <c r="B56" s="8"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="8"/>
-      <c r="I56" s="11"/>
-    </row>
-    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="12"/>
-      <c r="I57" s="15"/>
-    </row>
-    <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="8"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="8"/>
-      <c r="I58" s="11"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="12"/>
@@ -2435,60 +2730,2028 @@
       <c r="I59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="8"/>
-      <c r="B60" s="8"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="8"/>
-      <c r="I60" s="11"/>
+      <c r="A60" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F60" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12"/>
-      <c r="B61" s="12"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="13"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="15"/>
+      <c r="A61" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B61" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E61" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G61" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H61" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I61" s="15" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="8"/>
-      <c r="B62" s="8"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="8"/>
-      <c r="I62" s="11"/>
+      <c r="A62" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F62" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H62" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I62" s="11" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="12"/>
-      <c r="B63" s="12"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="13"/>
-      <c r="H63" s="12"/>
-      <c r="I63" s="15"/>
+      <c r="A63" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D63" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E63" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F63" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G63" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I63" s="15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F64" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I64" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E65" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F65" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G65" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H65" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="I65" s="15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12"/>
+      <c r="B66" s="12"/>
+      <c r="C66" s="13"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="14"/>
+      <c r="G66" s="13"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="15"/>
+    </row>
+    <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E67" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F67" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I67" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D68" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E68" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F68" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G68" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H68" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I68" s="15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H87" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G100" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H102" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H103" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I103" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H104" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H105" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I105" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H106" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H107" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I107" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H109" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I109" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H110" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I110" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G111" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H111" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I111" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H113" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I113" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H114" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I114" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H115" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I115" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G116" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H116" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H117" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I117" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I118" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="I121" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I123" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G124" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I124" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I125" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G126" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I126" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G128" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I128" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H130" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I130" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H131" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I131" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G132" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H132" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="I132" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G133" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H133" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I133" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G134" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H134" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I134" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G135" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H135" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I135" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E136" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G136" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H136" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I136" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G137" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H137" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I137" s="1" t="s">
+        <v>212</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C19:C22 C28:C31 C34:C36 C46:C63" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C19:C22 C28:C31 C34:C36 C48:C68" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E19:E22 E28:E31 E34:E36 E46:E63" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E19:E22 E28:E31 E34:E36 E48:E68" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F11 F19:F22 F28:F31 F34:F36 F46:F63" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F11 F19:F22 F28:F31 F34:F36 F48:F68" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2523,89 +4786,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>104</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>105</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>106</v>
+        <v>215</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>107</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>108</v>
+        <v>217</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>109</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>110</v>
+        <v>219</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>111</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>112</v>
+        <v>221</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>113</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>114</v>
+        <v>223</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>115</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>116</v>
+        <v>225</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>117</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>118</v>
+        <v>227</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>119</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>120</v>
+        <v>229</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>121</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>122</v>
+        <v>231</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>123</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>124</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2613,7 +4876,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>125</v>
+        <v>234</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -2628,10 +4891,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>126</v>
+        <v>235</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>127</v>
+        <v>236</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>16</v>
@@ -2639,245 +4902,245 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>129</v>
+        <v>238</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>132</v>
+        <v>241</v>
       </c>
       <c r="H17" s="12" t="s">
         <v>20</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>133</v>
+        <v>242</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>134</v>
+        <v>243</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>135</v>
+        <v>244</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>136</v>
+        <v>245</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>138</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>139</v>
+        <v>248</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>135</v>
+        <v>244</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>20</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>140</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>141</v>
+        <v>250</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>142</v>
+        <v>251</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>143</v>
+        <v>252</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>144</v>
+        <v>253</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>135</v>
+        <v>244</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>136</v>
+        <v>245</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>145</v>
+        <v>254</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>74</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>146</v>
+        <v>255</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>147</v>
+        <v>256</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>34</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>148</v>
+        <v>257</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>149</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>150</v>
+        <v>259</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>147</v>
+        <v>256</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>132</v>
+        <v>241</v>
       </c>
       <c r="H23" s="12" t="s">
         <v>20</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>151</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>150</v>
+        <v>259</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>152</v>
+        <v>261</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>135</v>
+        <v>244</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>153</v>
+        <v>262</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>154</v>
+        <v>263</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>150</v>
+        <v>259</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>155</v>
+        <v>264</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>156</v>
+        <v>265</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>157</v>
+        <v>266</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>158</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -2907,39 +5170,39 @@
         <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>145</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>159</v>
+        <v>268</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>160</v>
+        <v>269</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>161</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>162</v>
+        <v>271</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>137</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>163</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2949,27 +5212,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>164</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>142</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>165</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>166</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>167</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>